<commit_message>
fix: replace internal Gnumbers in Excel template files
</commit_message>
<xml_diff>
--- a/examples/LargeDrugCombo_Goetz_Cancers_2024/raw_data/P41.Belva.mtx17.template.xlsx
+++ b/examples/LargeDrugCombo_Goetz_Cancers_2024/raw_data/P41.Belva.mtx17.template.xlsx
@@ -66,22 +66,22 @@
     <t>P</t>
   </si>
   <si>
-    <t>G03083045.23-1</t>
+    <t>G00103</t>
   </si>
   <si>
-    <t>G00050939.150-10</t>
+    <t>G00105</t>
   </si>
   <si>
-    <t>G00044364.1-13</t>
+    <t>G00104</t>
   </si>
   <si>
-    <t xml:space="preserve">G03083045.23-1</t>
+    <t xml:space="preserve">G00103</t>
   </si>
   <si>
-    <t xml:space="preserve">G00044364.1-13</t>
+    <t xml:space="preserve">G00104</t>
   </si>
   <si>
-    <t xml:space="preserve">G00050939.150-10</t>
+    <t xml:space="preserve">G00105</t>
   </si>
   <si>
     <t xml:space="preserve">vehicle</t>

</xml_diff>